<commit_message>
Aggiornato treno 637 e capolinea Carnate Usmate in dir39
</commit_message>
<xml_diff>
--- a/direttrici/direttrici.xlsx
+++ b/direttrici/direttrici.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tommaso\.gemini\antigravity\scratch\monitor_treni\direttrici\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E32036ED-CA52-4D23-8F25-018F3A07E2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2611DF40-8347-4319-A5E6-94459FE8759C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6C15CDBC-8405-45FA-BA7F-E008D9D76093}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="85">
   <si>
     <t>Novara - Milano Passante - Treviglio</t>
   </si>
@@ -294,9 +294,6 @@
   </si>
   <si>
     <t>su 40</t>
-  </si>
-  <si>
-    <t>CHECK</t>
   </si>
 </sst>
 </file>
@@ -1122,9 +1119,6 @@
       <c r="D33" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>85</v>
-      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34">
@@ -1171,9 +1165,6 @@
       </c>
       <c r="D37" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
dir 27 e 28
</commit_message>
<xml_diff>
--- a/direttrici/direttrici.xlsx
+++ b/direttrici/direttrici.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tommaso\.gemini\antigravity\scratch\monitor_treni\direttrici\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B272CA1-38DE-403E-B5C9-DFE7D203FD92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC9087E7-2038-4621-9A39-B0F476807880}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6C15CDBC-8405-45FA-BA7F-E008D9D76093}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="87">
   <si>
     <t>Novara - Milano Passante - Treviglio</t>
   </si>
@@ -297,6 +297,9 @@
   </si>
   <si>
     <t>SOLO BUS</t>
+  </si>
+  <si>
+    <t>CHECK</t>
   </si>
 </sst>
 </file>
@@ -318,7 +321,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -334,6 +337,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -385,7 +394,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -395,6 +404,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -950,7 +960,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
@@ -961,7 +971,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>18</v>
       </c>
@@ -975,7 +985,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="19" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>19</v>
       </c>
@@ -989,7 +999,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
@@ -1000,7 +1010,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>21</v>
       </c>
@@ -1014,7 +1024,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
@@ -1025,7 +1035,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="23" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>23</v>
       </c>
@@ -1039,7 +1049,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="24" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>24</v>
       </c>
@@ -1053,7 +1063,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
@@ -1064,7 +1074,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>26</v>
       </c>
@@ -1075,29 +1085,41 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27">
+    <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="2">
         <v>27</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28">
+      <c r="D27" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="2">
         <v>28</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D28" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>29</v>
       </c>
@@ -1108,7 +1130,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
@@ -1119,7 +1141,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>31</v>
       </c>
@@ -1130,7 +1152,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>32</v>
       </c>
@@ -1251,7 +1273,7 @@
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D43" s="4">
         <f>COUNTIF(D1:D42,"ok")</f>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E43" s="5" t="s">
         <v>84</v>

</xml_diff>

<commit_message>
dir 32 e 40
</commit_message>
<xml_diff>
--- a/direttrici/direttrici.xlsx
+++ b/direttrici/direttrici.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tommaso\.gemini\antigravity\scratch\monitor_treni\direttrici\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04D073B-EA73-4E1E-8494-7EFA4E6F3A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C16334B7-D0C8-4245-BBAE-4C90675E11B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6C15CDBC-8405-45FA-BA7F-E008D9D76093}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="88">
   <si>
     <t>Novara - Milano Passante - Treviglio</t>
   </si>
@@ -297,6 +297,12 @@
   </si>
   <si>
     <t>SOLO BUS</t>
+  </si>
+  <si>
+    <t>non si capice</t>
+  </si>
+  <si>
+    <t>CHECK</t>
   </si>
 </sst>
 </file>
@@ -318,7 +324,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -334,6 +340,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -385,7 +397,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -395,6 +407,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -735,7 +748,7 @@
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="97.44140625" customWidth="1"/>
     <col min="3" max="3" width="14.44140625" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -950,7 +963,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
@@ -961,7 +974,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>18</v>
       </c>
@@ -975,7 +988,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="19" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>19</v>
       </c>
@@ -989,7 +1002,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
@@ -1000,7 +1013,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>21</v>
       </c>
@@ -1014,7 +1027,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
@@ -1025,7 +1038,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="23" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>23</v>
       </c>
@@ -1039,7 +1052,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="24" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>24</v>
       </c>
@@ -1053,7 +1066,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
@@ -1064,18 +1077,21 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26">
+    <row r="26" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="7">
         <v>26</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="7" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="E26" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>27</v>
       </c>
@@ -1089,7 +1105,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="28" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>28</v>
       </c>
@@ -1103,18 +1119,21 @@
         <v>83</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29">
+    <row r="29" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="7">
         <v>29</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="7" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E29" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
@@ -1125,7 +1144,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>31</v>
       </c>
@@ -1136,15 +1155,21 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32">
+    <row r="32" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="2">
         <v>32</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="2" t="s">
         <v>39</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1227,15 +1252,21 @@
         <v>83</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40">
+    <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="2">
         <v>40</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C40" s="2" t="s">
         <v>61</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
@@ -1257,7 +1288,7 @@
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D43" s="4">
         <f>COUNTIF(D1:D42,"ok")</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E43" s="5" t="s">
         <v>84</v>

</xml_diff>

<commit_message>
dir 2 e 5
</commit_message>
<xml_diff>
--- a/direttrici/direttrici.xlsx
+++ b/direttrici/direttrici.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tommaso\.gemini\antigravity\scratch\monitor_treni\direttrici\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2593D6DE-D0E0-4D59-B3F7-FDFD070D2809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{295B0E76-43C1-410D-809E-270ABAE2E0BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6C15CDBC-8405-45FA-BA7F-E008D9D76093}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="86">
   <si>
     <t>Novara - Milano Passante - Treviglio</t>
   </si>
@@ -272,18 +272,9 @@
     <t>tilo</t>
   </si>
   <si>
-    <t>Biasca - Bellinzona - Lugano - Varese - Malpensa</t>
-  </si>
-  <si>
-    <t>S50</t>
-  </si>
-  <si>
     <t>Luino - Gallarate – Milano / Cadenazzo - Luino - Gallarate</t>
   </si>
   <si>
-    <t>R12 / S30</t>
-  </si>
-  <si>
     <t>Como - Milano - Rho / Como - Mendrisio - Varese / Chiasso - Milano Centrale</t>
   </si>
   <si>
@@ -293,13 +284,19 @@
     <t>ok</t>
   </si>
   <si>
-    <t>su 39</t>
-  </si>
-  <si>
     <t>SOLO BUS</t>
   </si>
   <si>
     <t>non si capice</t>
+  </si>
+  <si>
+    <t>R21 / S30</t>
+  </si>
+  <si>
+    <t>su 38</t>
+  </si>
+  <si>
+    <t>CHECK</t>
   </si>
 </sst>
 </file>
@@ -347,21 +344,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -394,7 +382,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -402,7 +390,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
@@ -739,7 +726,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E6BE5C4-52B3-4A8B-9EE7-686436176D81}">
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -759,18 +746,24 @@
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>71</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -795,18 +788,24 @@
         <v>5</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C5" t="s">
-        <v>80</v>
+      <c r="D5" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -814,13 +813,13 @@
         <v>6</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -834,7 +833,7 @@
         <v>51</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -848,7 +847,7 @@
         <v>63</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -862,7 +861,7 @@
         <v>21</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -876,7 +875,7 @@
         <v>23</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -901,21 +900,21 @@
         <v>11</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="6">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="5">
         <v>13</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E13" s="6" t="s">
-        <v>85</v>
+      <c r="E13" s="5" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -929,7 +928,7 @@
         <v>13</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -943,7 +942,7 @@
         <v>3</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -957,7 +956,7 @@
         <v>29</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -982,7 +981,7 @@
         <v>16</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -996,7 +995,7 @@
         <v>17</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -1021,7 +1020,7 @@
         <v>47</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
@@ -1046,7 +1045,7 @@
         <v>53</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1060,7 +1059,7 @@
         <v>41</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -1074,18 +1073,18 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="7">
+    <row r="26" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="6">
         <v>26</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="E26" s="7" t="s">
-        <v>86</v>
+      <c r="E26" s="6" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1099,7 +1098,7 @@
         <v>45</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1113,21 +1112,21 @@
         <v>43</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="7">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="6">
         <v>29</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="E29" s="7" t="s">
-        <v>86</v>
+      <c r="E29" s="6" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -1163,7 +1162,7 @@
         <v>39</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="33" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1177,7 +1176,7 @@
         <v>9</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
@@ -1224,7 +1223,7 @@
         <v>59</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="38" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1238,7 +1237,7 @@
         <v>65</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="39" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1252,37 +1251,26 @@
         <v>61</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="3">
-        <v>42</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D41" s="4">
-        <f>COUNTIF(D1:D40,"ok")</f>
-        <v>23</v>
-      </c>
-      <c r="E41" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D40" s="3">
+        <f>COUNTIF(D1:D39,"ok")</f>
+        <v>25</v>
+      </c>
+      <c r="E40" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
         <v>76</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B42" t="s">
         <v>74</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C42" t="s">
         <v>75</v>
       </c>
     </row>

</xml_diff>

<commit_message>
dir 3 e 11
</commit_message>
<xml_diff>
--- a/direttrici/direttrici.xlsx
+++ b/direttrici/direttrici.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tommaso\.gemini\antigravity\scratch\monitor_treni\direttrici\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FA86DE3-2974-44D6-895D-054212A253C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A39EAB66-88C4-4DA5-9193-E6F170A23085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6C15CDBC-8405-45FA-BA7F-E008D9D76093}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="86">
   <si>
     <t>Novara - Milano Passante - Treviglio</t>
   </si>
@@ -131,18 +131,9 @@
     <t>R6</t>
   </si>
   <si>
-    <t>Domodossola - Milano / Domodossola - Arona - Gallarate - Milano / Laveno – Sesto Calende</t>
-  </si>
-  <si>
-    <t>RE4 / R23 / R24</t>
-  </si>
-  <si>
     <t>Bergamo - Brescia / Lecco - Bergamo</t>
   </si>
   <si>
-    <t>R1 / R7</t>
-  </si>
-  <si>
     <t>Mortara - Alessandria / Mortara - Milano</t>
   </si>
   <si>
@@ -294,6 +285,18 @@
   </si>
   <si>
     <t>su 38</t>
+  </si>
+  <si>
+    <t>Domodossola - Milano / Domodossola - Arona - Gallarate - Milano</t>
+  </si>
+  <si>
+    <t>RE4 / R23</t>
+  </si>
+  <si>
+    <t>CHECK</t>
+  </si>
+  <si>
+    <t>R1</t>
   </si>
 </sst>
 </file>
@@ -743,7 +746,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -751,24 +754,30 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" t="s">
-        <v>31</v>
+      <c r="B3" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -782,7 +791,7 @@
         <v>5</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -790,13 +799,13 @@
         <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -804,13 +813,13 @@
         <v>6</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -818,13 +827,13 @@
         <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -832,13 +841,13 @@
         <v>8</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -852,7 +861,7 @@
         <v>21</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -866,18 +875,24 @@
         <v>23</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2">
         <v>11</v>
       </c>
-      <c r="B11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" t="s">
-        <v>33</v>
+      <c r="B11" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -891,7 +906,7 @@
         <v>11</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -899,13 +914,13 @@
         <v>13</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -919,7 +934,7 @@
         <v>13</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -933,7 +948,7 @@
         <v>3</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -947,7 +962,7 @@
         <v>29</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -972,7 +987,7 @@
         <v>16</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -986,7 +1001,7 @@
         <v>17</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -1005,13 +1020,13 @@
         <v>21</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
@@ -1019,10 +1034,10 @@
         <v>22</v>
       </c>
       <c r="B22" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C22" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1030,13 +1045,13 @@
         <v>23</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1044,13 +1059,13 @@
         <v>24</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -1058,10 +1073,10 @@
         <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.3">
@@ -1069,13 +1084,13 @@
         <v>26</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1083,13 +1098,13 @@
         <v>27</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1097,13 +1112,13 @@
         <v>28</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="29" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.3">
@@ -1111,13 +1126,13 @@
         <v>29</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -1125,10 +1140,10 @@
         <v>30</v>
       </c>
       <c r="B30" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C30" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
@@ -1147,13 +1162,13 @@
         <v>32</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1167,7 +1182,7 @@
         <v>9</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
@@ -1175,10 +1190,10 @@
         <v>34</v>
       </c>
       <c r="B34" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C34" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
@@ -1197,10 +1212,10 @@
         <v>36</v>
       </c>
       <c r="B36" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C36" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1208,13 +1223,13 @@
         <v>37</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="38" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1222,13 +1237,13 @@
         <v>39</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="39" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1236,37 +1251,38 @@
         <v>40</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D40" s="3">
         <f>COUNTIF(D1:D39,"ok")</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B42" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C42" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Aggiornato README.md con note legali su diritti d'autore e proprieta del codice
</commit_message>
<xml_diff>
--- a/direttrici/direttrici.xlsx
+++ b/direttrici/direttrici.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tommaso\.gemini\antigravity\scratch\monitor_treni\direttrici\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57387E73-39B5-4FBB-A785-7B1808B198C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B73C9E7C-4920-4181-B86E-B0DFA80802A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6C15CDBC-8405-45FA-BA7F-E008D9D76093}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="86">
   <si>
     <t>Novara - Milano Passante - Treviglio</t>
   </si>
@@ -969,6 +969,9 @@
       <c r="C17" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="D17" s="1" t="s">
+        <v>77</v>
+      </c>
       <c r="E17" s="5" t="s">
         <v>85</v>
       </c>
@@ -1260,7 +1263,7 @@
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D40" s="2">
         <f>COUNTIF(D1:D39,"ok")</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>81</v>

</xml_diff>